<commit_message>
Automating update for plant 52152 to correctly allocate heat input and emissions to unit 6RB, adding check for outliers in plant level emission rates using z-scores
</commit_message>
<xml_diff>
--- a/data/static_tables/manual_corrections.xlsx
+++ b/data/static_tables/manual_corrections.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\projects\eGrid\production_model\users\gofortht\data\static_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD33EAC3-267A-4AFE-8CEA-24A070777F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{053205CE-D372-4165-AD7C-5ECADBBADABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="3" xr2:uid="{FA61C6A3-A5F8-4301-A228-D222830EB6CC}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" firstSheet="1" activeTab="3" xr2:uid="{FA61C6A3-A5F8-4301-A228-D222830EB6CC}"/>
   </bookViews>
   <sheets>
     <sheet name="epa_clean" sheetId="5" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="55">
   <si>
     <t>plant_id</t>
   </si>
@@ -150,73 +150,7 @@
     <t>3</t>
   </si>
   <si>
-    <t>52152</t>
-  </si>
-  <si>
-    <t>6RB</t>
-  </si>
-  <si>
     <t>ST</t>
-  </si>
-  <si>
-    <t>heat_input</t>
-  </si>
-  <si>
-    <t>6413476.992</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 2383097.20 </t>
-  </si>
-  <si>
-    <t>heat_input_oz</t>
-  </si>
-  <si>
-    <t>nox_mass</t>
-  </si>
-  <si>
-    <t>272.69</t>
-  </si>
-  <si>
-    <t>nox_oz_mass</t>
-  </si>
-  <si>
-    <t>97.016</t>
-  </si>
-  <si>
-    <t>so2_mass</t>
-  </si>
-  <si>
-    <t>1272.5545</t>
-  </si>
-  <si>
-    <t>co2_mass</t>
-  </si>
-  <si>
-    <t>608148.783</t>
-  </si>
-  <si>
-    <t>heat_input_source</t>
-  </si>
-  <si>
-    <t>EIA Prime Mover-level Data</t>
-  </si>
-  <si>
-    <t>heat_input_oz_source</t>
-  </si>
-  <si>
-    <t>nox_source</t>
-  </si>
-  <si>
-    <t>Estimated using emissions factor</t>
-  </si>
-  <si>
-    <t>nox_oz_source</t>
-  </si>
-  <si>
-    <t>so2_source</t>
-  </si>
-  <si>
-    <t>co2_source</t>
   </si>
   <si>
     <t>operating_status</t>
@@ -697,10 +631,10 @@
         <v>10154</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -734,10 +668,10 @@
         <v>60910</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -889,7 +823,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C1A8242-D17A-4DAB-8319-EC8C1026D049}">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="8.140625" style="3" bestFit="1" customWidth="1"/>
@@ -1003,7 +937,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="D9" t="s">
         <v>10</v>
@@ -1011,7 +945,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
@@ -1120,324 +1054,120 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C18" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D18" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" t="s">
-        <v>38</v>
-      </c>
       <c r="D19" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C20" t="s">
-        <v>38</v>
-      </c>
       <c r="D20" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C21" t="s">
-        <v>38</v>
-      </c>
       <c r="D21" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C22" t="s">
-        <v>38</v>
-      </c>
       <c r="D22" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>37</v>
+        <v>46</v>
+      </c>
+      <c r="B23" t="s">
+        <v>53</v>
       </c>
       <c r="C23" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="D23" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="C24" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="D24" t="s">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C25" t="s">
-        <v>38</v>
-      </c>
-      <c r="D25" t="s">
-        <v>53</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C26" t="s">
-        <v>38</v>
-      </c>
-      <c r="D26" t="s">
-        <v>54</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C27" t="s">
-        <v>38</v>
-      </c>
-      <c r="D27" t="s">
-        <v>56</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C28" t="s">
-        <v>38</v>
-      </c>
-      <c r="D28" t="s">
-        <v>57</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C29" t="s">
-        <v>38</v>
-      </c>
-      <c r="D29" t="s">
-        <v>58</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C30" t="s">
-        <v>30</v>
-      </c>
-      <c r="D30" t="s">
-        <v>12</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C31" t="s">
-        <v>38</v>
-      </c>
-      <c r="D31" t="s">
-        <v>73</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C32" t="s">
-        <v>38</v>
-      </c>
-      <c r="D32" t="s">
-        <v>73</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C33" t="s">
-        <v>38</v>
-      </c>
-      <c r="D33" t="s">
-        <v>73</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B34" t="s">
-        <v>72</v>
-      </c>
-      <c r="C34" t="s">
-        <v>38</v>
-      </c>
-      <c r="D34" t="s">
-        <v>73</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B35" t="s">
-        <v>75</v>
-      </c>
-      <c r="C35" t="s">
-        <v>13</v>
-      </c>
-      <c r="D35" t="s">
-        <v>12</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C36" t="s">
-        <v>13</v>
-      </c>
-      <c r="D36" t="s">
-        <v>12</v>
-      </c>
-      <c r="E36" s="3" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1514,7 +1244,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>67</v>
+        <v>45</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>17</v>
@@ -1525,7 +1255,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>67</v>
+        <v>45</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>18</v>

</xml_diff>